<commit_message>
Add 12 VAC voltage input support
</commit_message>
<xml_diff>
--- a/bom/ADE9000_Breakout_BOM.xlsx
+++ b/bom/ADE9000_Breakout_BOM.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TerminalBlock_4Ucon:TerminalBlock_4Ucon_1x02_P3.50mm_Horizontal</t>
+          <t>ADE9000-Local:TerminalBlock_4Ucon_1x02_P3.50mm_Horizontal_ADE9000</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -746,47 +746,47 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R21, R22, R23, R24, R25, R26</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ADE9000</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Package_DFN_QFN:QFN-40-1EP_6x6mm_P0.5mm_EP4.27x4.27mm</t>
+          <t>Resistor_SMD:R_0402_1005Metric</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ADE9000ACPZ</t>
+          <t>RC0402FR-07100KL</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=ADE9000ACPZ</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-07100KL</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=ADE9000ACPZ</t>
+          <t>https://www.mouser.com/c/?q=RC0402FR-07100KL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>ADE9000 polyphase energy and power quality monitoring IC, CP-40-7 LFCSP</t>
+          <t>100 kOhm 1% 0402 voltage-divider high-side resistor</t>
         </is>
       </c>
     </row>
@@ -798,45 +798,149 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>R27, R28, R29, R30, R31, R32</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.49k</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Resistor_SMD:R_0402_1005Metric</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>RC0402FR-072K49L</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-072K49L</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/c/?q=RC0402FR-072K49L</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2.49 kOhm 1% 0402 voltage-divider shunt resistor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ADE9000</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Package_DFN_QFN:QFN-40-1EP_6x6mm_P0.5mm_EP4.27x4.27mm</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ADE9000ACPZ</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.digikey.com/en/products/result?keywords=ADE9000ACPZ</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/c/?q=ADE9000ACPZ</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>ADE9000 polyphase energy and power quality monitoring IC, CP-40-7 LFCSP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>24.576MHz</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Crystal:Crystal_SMD_3225-4Pin_3.2x2.5mm</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>ECS Inc.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>ECS-245.7-12-33Q-JES-TR</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>https://www.digikey.com/en/products/result?keywords=ECS-245.7-12-33Q-JES-TR</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>https://www.mouser.com/c/?q=ECS-245.7-12-33Q-JES-TR</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>24.576 MHz 3.2 x 2.5 mm SMD crystal</t>
         </is>

</xml_diff>

<commit_message>
Use 0603 passives for hand assembly
</commit_message>
<xml_diff>
--- a/bom/ADE9000_Breakout_BOM.xlsx
+++ b/bom/ADE9000_Breakout_BOM.xlsx
@@ -137,7 +137,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0402_1005Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -147,22 +147,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>GRM155R71A104KA01D</t>
+          <t>GRM188R71A104KA61D</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=GRM155R71A104KA01D</t>
+          <t>https://www.digikey.com/en/products/result?keywords=GRM188R71A104KA61D</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=GRM155R71A104KA01D</t>
+          <t>https://www.mouser.com/c/?q=GRM188R71A104KA61D</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>100 nF 10 V X7R 0402 ceramic capacitor</t>
+          <t>100 nF 10 V X7R 0603 ceramic capacitor</t>
         </is>
       </c>
     </row>
@@ -241,7 +241,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0402_1005Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -251,22 +251,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>GRM1555C1H160JA01D</t>
+          <t>GRM1885C1H160JA01D</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=GRM1555C1H160JA01D</t>
+          <t>https://www.digikey.com/en/products/result?keywords=GRM1885C1H160JA01D</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=GRM1555C1H160JA01D</t>
+          <t>https://www.mouser.com/c/?q=GRM1885C1H160JA01D</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>16 pF 50 V C0G/NP0 0402 ceramic capacitor</t>
+          <t>16 pF 50 V C0G/NP0 0603 ceramic capacitor</t>
         </is>
       </c>
     </row>
@@ -293,7 +293,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0402_1005Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -303,22 +303,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>GRM155R61A105KE15D</t>
+          <t>GRM188R61A105KA61D</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=GRM155R61A105KE15D</t>
+          <t>https://www.digikey.com/en/products/result?keywords=GRM188R61A105KA61D</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=GRM155R61A105KE15D</t>
+          <t>https://www.mouser.com/c/?q=GRM188R61A105KA61D</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1 uF 10 V X5R 0402 ceramic capacitor</t>
+          <t>1 uF 10 V X5R 0603 ceramic capacitor</t>
         </is>
       </c>
     </row>
@@ -345,7 +345,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Capacitor_SMD:C_0402_1005Metric</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -355,22 +355,22 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>GRM155R71H223KA12D</t>
+          <t>GRM188R71H223KA01D</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=GRM155R71H223KA12D</t>
+          <t>https://www.digikey.com/en/products/result?keywords=GRM188R71H223KA01D</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=GRM155R71H223KA12D</t>
+          <t>https://www.mouser.com/c/?q=GRM188R71H223KA01D</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>22 nF 50 V X7R 0402 ceramic capacitor</t>
+          <t>22 nF 50 V X7R 0603 ceramic capacitor</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0402_1005Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -615,22 +615,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-0710KL</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=RC0402FR-0710KL</t>
+          <t>https://www.mouser.com/c/?q=RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>10 kOhm 1% 0402 thick-film resistor</t>
+          <t>10 kOhm 1% 0603 thick-film resistor</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0402_1005Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -667,22 +667,22 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-071KL</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0603FR-071KL</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=RC0402FR-071KL</t>
+          <t>https://www.mouser.com/c/?q=RC0603FR-071KL</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1 kOhm 1% 0402 thick-film resistor</t>
+          <t>1 kOhm 1% 0603 thick-film resistor</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0402_1005Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -719,22 +719,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>RC0402FR-072R4L</t>
+          <t>RC0603FR-072R4L</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-072R4L</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0603FR-072R4L</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=RC0402FR-072R4L</t>
+          <t>https://www.mouser.com/c/?q=RC0603FR-072R4L</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2.4 Ohm 1% 0402 thick-film burden resistor</t>
+          <t>2.4 Ohm 1% 0603 thick-film burden resistor</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0402_1005Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -771,22 +771,22 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>RC0402FR-07100KL</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-07100KL</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=RC0402FR-07100KL</t>
+          <t>https://www.mouser.com/c/?q=RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>100 kOhm 1% 0402 voltage-divider high-side resistor</t>
+          <t>100 kOhm 1% 0603 voltage-divider high-side resistor</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Resistor_SMD:R_0402_1005Metric</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -823,22 +823,22 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>RC0402FR-072K49L</t>
+          <t>RC0603FR-072K49L</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=RC0402FR-072K49L</t>
+          <t>https://www.digikey.com/en/products/result?keywords=RC0603FR-072K49L</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=RC0402FR-072K49L</t>
+          <t>https://www.mouser.com/c/?q=RC0603FR-072K49L</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2.49 kOhm 1% 0402 voltage-divider shunt resistor</t>
+          <t>2.49 kOhm 1% 0603 voltage-divider shunt resistor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add selectable ADE9000 power modes
Add ATM-style PM0/PM1 solder bridges, regenerate the routed board and BOM, and publish populated isometric renders in the README.\n\nCo-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bom/ADE9000_Breakout_BOM.xlsx
+++ b/bom/ADE9000_Breakout_BOM.xlsx
@@ -142,27 +142,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>GRM188R71A104KA61D</t>
+          <t>CC0603KPX7R0BB104</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=GRM188R71A104KA61D</t>
+          <t>https://www.digikey.com.au/en/products/detail/yageo/CC0603KPX7R0BB104/29291093</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/?q=GRM188R71A104KA61D</t>
+          <t>https://www.mouser.com/c/?q=CC0603KPX7R0BB104</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>100 nF 10 V X7R 0603 ceramic capacitor</t>
+          <t>100 nF 100 V 10% X7R 0603 ceramic capacitor</t>
         </is>
       </c>
     </row>

</xml_diff>